<commit_message>
跟随英雄联盟更新的例行更新【A Regular Update following the New LoL Patch】
更新了离线数据资源文件。（最近更新：2024年4月2日。）
Updated offline data resources. (Latest update: 2024-04-02.)
此外，更新了斯卡纳的称号。
Besides, updated the title of Skarner.
</commit_message>
<xml_diff>
--- a/available-bots.xlsx
+++ b/available-bots.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\19250\Documents\GitHub\LoL-DIY-Programs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58840920-0442-4B80-994E-A652E236E095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFB7631B-DA4C-4838-8639-27E5AA780505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{79371658-E0FE-43C3-8A19-9910316D4D47}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{79371658-E0FE-43C3-8A19-9910316D4D47}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -421,9 +421,6 @@
     <t>机械公敌</t>
   </si>
   <si>
-    <t>水晶先锋</t>
-  </si>
-  <si>
     <t>大发明家</t>
   </si>
   <si>
@@ -1049,6 +1046,9 @@
   </si>
   <si>
     <t>Smolder</t>
+  </si>
+  <si>
+    <t>上古领主</t>
   </si>
 </sst>
 </file>
@@ -1116,9 +1116,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 主题">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1156,7 +1156,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1262,7 +1262,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1404,7 +1404,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1420,10 +1420,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>325</v>
+      </c>
+      <c r="C1" t="s">
         <v>326</v>
-      </c>
-      <c r="C1" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -1621,7 +1621,7 @@
         <v>35</v>
       </c>
       <c r="C19" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -1654,7 +1654,7 @@
         <v>40</v>
       </c>
       <c r="C22" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
@@ -1742,7 +1742,7 @@
         <v>55</v>
       </c>
       <c r="C30" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
@@ -1830,7 +1830,7 @@
         <v>72</v>
       </c>
       <c r="C38" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
@@ -1938,10 +1938,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>325</v>
+      </c>
+      <c r="C1" t="s">
         <v>326</v>
-      </c>
-      <c r="C1" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -1963,7 +1963,7 @@
         <v>103</v>
       </c>
       <c r="C3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -1985,7 +1985,7 @@
         <v>104</v>
       </c>
       <c r="C5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -1996,7 +1996,7 @@
         <v>105</v>
       </c>
       <c r="C6" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -2007,7 +2007,7 @@
         <v>106</v>
       </c>
       <c r="C7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -2095,7 +2095,7 @@
         <v>109</v>
       </c>
       <c r="C15" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -2216,7 +2216,7 @@
         <v>35</v>
       </c>
       <c r="C26" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
@@ -2249,7 +2249,7 @@
         <v>40</v>
       </c>
       <c r="C29" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
@@ -2260,7 +2260,7 @@
         <v>110</v>
       </c>
       <c r="C30" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
@@ -2271,7 +2271,7 @@
         <v>111</v>
       </c>
       <c r="C31" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
@@ -2282,7 +2282,7 @@
         <v>112</v>
       </c>
       <c r="C32" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
@@ -2293,7 +2293,7 @@
         <v>113</v>
       </c>
       <c r="C33" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
@@ -2370,7 +2370,7 @@
         <v>118</v>
       </c>
       <c r="C40" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
@@ -2381,7 +2381,7 @@
         <v>119</v>
       </c>
       <c r="C41" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
@@ -2392,7 +2392,7 @@
         <v>120</v>
       </c>
       <c r="C42" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
@@ -2414,7 +2414,7 @@
         <v>123</v>
       </c>
       <c r="C44" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
@@ -2425,7 +2425,7 @@
         <v>55</v>
       </c>
       <c r="C45" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
@@ -2447,7 +2447,7 @@
         <v>125</v>
       </c>
       <c r="C47" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
@@ -2458,7 +2458,7 @@
         <v>126</v>
       </c>
       <c r="C48" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
@@ -2477,10 +2477,10 @@
         <v>74</v>
       </c>
       <c r="B50" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C50" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
@@ -2510,10 +2510,10 @@
         <v>78</v>
       </c>
       <c r="B53" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C53" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
@@ -2532,10 +2532,10 @@
         <v>82</v>
       </c>
       <c r="B55" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C55" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
@@ -2543,10 +2543,10 @@
         <v>83</v>
       </c>
       <c r="B56" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C56" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
@@ -2554,10 +2554,10 @@
         <v>84</v>
       </c>
       <c r="B57" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C57" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
@@ -2565,10 +2565,10 @@
         <v>85</v>
       </c>
       <c r="B58" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C58" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
@@ -2598,10 +2598,10 @@
         <v>90</v>
       </c>
       <c r="B61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C61" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
@@ -2612,7 +2612,7 @@
         <v>72</v>
       </c>
       <c r="C62" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
@@ -2653,10 +2653,10 @@
         <v>103</v>
       </c>
       <c r="B66" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C66" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
@@ -2675,10 +2675,10 @@
         <v>105</v>
       </c>
       <c r="B68" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C68" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
@@ -2686,10 +2686,10 @@
         <v>106</v>
       </c>
       <c r="B69" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C69" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
@@ -2697,10 +2697,10 @@
         <v>110</v>
       </c>
       <c r="B70" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C70" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
@@ -2708,10 +2708,10 @@
         <v>111</v>
       </c>
       <c r="B71" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C71" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
@@ -2719,10 +2719,10 @@
         <v>112</v>
       </c>
       <c r="B72" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C72" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
@@ -2730,10 +2730,10 @@
         <v>113</v>
       </c>
       <c r="B73" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C73" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
@@ -2752,10 +2752,10 @@
         <v>117</v>
       </c>
       <c r="B75" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C75" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
@@ -2763,10 +2763,10 @@
         <v>120</v>
       </c>
       <c r="B76" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C76" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.2">
@@ -2774,10 +2774,10 @@
         <v>121</v>
       </c>
       <c r="B77" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C77" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.2">
@@ -2796,10 +2796,10 @@
         <v>127</v>
       </c>
       <c r="B79" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C79" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.2">
@@ -2807,10 +2807,10 @@
         <v>131</v>
       </c>
       <c r="B80" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C80" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
@@ -2829,10 +2829,10 @@
         <v>145</v>
       </c>
       <c r="B82" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C82" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.2">
@@ -2840,10 +2840,10 @@
         <v>147</v>
       </c>
       <c r="B83" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C83" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.2">
@@ -2851,10 +2851,10 @@
         <v>201</v>
       </c>
       <c r="B84" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C84" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.2">
@@ -2873,10 +2873,10 @@
         <v>254</v>
       </c>
       <c r="B86" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C86" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.2">
@@ -2884,10 +2884,10 @@
         <v>266</v>
       </c>
       <c r="B87" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C87" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
@@ -2895,10 +2895,10 @@
         <v>497</v>
       </c>
       <c r="B88" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C88" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
@@ -2906,10 +2906,10 @@
         <v>711</v>
       </c>
       <c r="B89" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C89" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.2">
@@ -2917,10 +2917,10 @@
         <v>875</v>
       </c>
       <c r="B90" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C90" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.2">
@@ -2928,10 +2928,10 @@
         <v>876</v>
       </c>
       <c r="B91" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C91" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.2">
@@ -2939,10 +2939,10 @@
         <v>888</v>
       </c>
       <c r="B92" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C92" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.2">
@@ -2950,10 +2950,10 @@
         <v>901</v>
       </c>
       <c r="B93" t="s">
+        <v>334</v>
+      </c>
+      <c r="C93" t="s">
         <v>335</v>
-      </c>
-      <c r="C93" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.2">
@@ -2961,10 +2961,10 @@
         <v>902</v>
       </c>
       <c r="B94" t="s">
+        <v>321</v>
+      </c>
+      <c r="C94" t="s">
         <v>322</v>
-      </c>
-      <c r="C94" t="s">
-        <v>323</v>
       </c>
     </row>
   </sheetData>
@@ -2987,10 +2987,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>325</v>
+      </c>
+      <c r="C1" t="s">
         <v>326</v>
-      </c>
-      <c r="C1" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -3012,7 +3012,7 @@
         <v>103</v>
       </c>
       <c r="C3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -3034,7 +3034,7 @@
         <v>104</v>
       </c>
       <c r="C5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -3045,7 +3045,7 @@
         <v>105</v>
       </c>
       <c r="C6" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -3056,7 +3056,7 @@
         <v>106</v>
       </c>
       <c r="C7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -3067,7 +3067,7 @@
         <v>107</v>
       </c>
       <c r="C8" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -3089,7 +3089,7 @@
         <v>89</v>
       </c>
       <c r="C10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -3144,7 +3144,7 @@
         <v>108</v>
       </c>
       <c r="C15" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -3177,7 +3177,7 @@
         <v>109</v>
       </c>
       <c r="C18" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -3331,7 +3331,7 @@
         <v>35</v>
       </c>
       <c r="C32" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
@@ -3364,7 +3364,7 @@
         <v>100</v>
       </c>
       <c r="C35" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
@@ -3386,7 +3386,7 @@
         <v>40</v>
       </c>
       <c r="C37" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
@@ -3397,7 +3397,7 @@
         <v>110</v>
       </c>
       <c r="C38" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
@@ -3408,7 +3408,7 @@
         <v>111</v>
       </c>
       <c r="C39" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
@@ -3419,7 +3419,7 @@
         <v>112</v>
       </c>
       <c r="C40" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
@@ -3430,7 +3430,7 @@
         <v>113</v>
       </c>
       <c r="C41" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
@@ -3441,7 +3441,7 @@
         <v>114</v>
       </c>
       <c r="C42" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
@@ -3452,7 +3452,7 @@
         <v>115</v>
       </c>
       <c r="C43" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
@@ -3463,7 +3463,7 @@
         <v>116</v>
       </c>
       <c r="C44" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
@@ -3507,7 +3507,7 @@
         <v>117</v>
       </c>
       <c r="C48" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
@@ -3551,7 +3551,7 @@
         <v>118</v>
       </c>
       <c r="C52" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
@@ -3562,7 +3562,7 @@
         <v>119</v>
       </c>
       <c r="C53" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
@@ -3573,7 +3573,7 @@
         <v>120</v>
       </c>
       <c r="C54" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
@@ -3595,7 +3595,7 @@
         <v>121</v>
       </c>
       <c r="C56" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
@@ -3606,7 +3606,7 @@
         <v>122</v>
       </c>
       <c r="C57" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
@@ -3617,7 +3617,7 @@
         <v>123</v>
       </c>
       <c r="C58" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
@@ -3628,7 +3628,7 @@
         <v>55</v>
       </c>
       <c r="C59" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
@@ -3650,7 +3650,7 @@
         <v>124</v>
       </c>
       <c r="C61" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
@@ -3661,7 +3661,7 @@
         <v>125</v>
       </c>
       <c r="C62" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
@@ -3672,7 +3672,7 @@
         <v>126</v>
       </c>
       <c r="C63" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
@@ -3691,10 +3691,10 @@
         <v>72</v>
       </c>
       <c r="B65" t="s">
-        <v>127</v>
+        <v>336</v>
       </c>
       <c r="C65" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
@@ -3702,10 +3702,10 @@
         <v>74</v>
       </c>
       <c r="B66" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C66" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
@@ -3746,10 +3746,10 @@
         <v>78</v>
       </c>
       <c r="B70" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C70" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
@@ -3757,10 +3757,10 @@
         <v>79</v>
       </c>
       <c r="B71" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C71" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
@@ -3768,10 +3768,10 @@
         <v>80</v>
       </c>
       <c r="B72" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C72" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
@@ -3790,10 +3790,10 @@
         <v>82</v>
       </c>
       <c r="B74" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C74" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
@@ -3801,10 +3801,10 @@
         <v>83</v>
       </c>
       <c r="B75" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C75" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
@@ -3812,10 +3812,10 @@
         <v>84</v>
       </c>
       <c r="B76" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C76" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.2">
@@ -3823,10 +3823,10 @@
         <v>85</v>
       </c>
       <c r="B77" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C77" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.2">
@@ -3856,10 +3856,10 @@
         <v>90</v>
       </c>
       <c r="B80" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C80" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
@@ -3867,10 +3867,10 @@
         <v>91</v>
       </c>
       <c r="B81" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C81" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.2">
@@ -3878,10 +3878,10 @@
         <v>92</v>
       </c>
       <c r="B82" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C82" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.2">
@@ -3892,7 +3892,7 @@
         <v>72</v>
       </c>
       <c r="C83" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.2">
@@ -3922,10 +3922,10 @@
         <v>101</v>
       </c>
       <c r="B86" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C86" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.2">
@@ -3944,10 +3944,10 @@
         <v>103</v>
       </c>
       <c r="B88" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C88" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
@@ -3966,10 +3966,10 @@
         <v>105</v>
       </c>
       <c r="B90" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C90" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.2">
@@ -3977,10 +3977,10 @@
         <v>106</v>
       </c>
       <c r="B91" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C91" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.2">
@@ -3988,10 +3988,10 @@
         <v>107</v>
       </c>
       <c r="B92" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C92" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.2">
@@ -3999,10 +3999,10 @@
         <v>110</v>
       </c>
       <c r="B93" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C93" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.2">
@@ -4010,10 +4010,10 @@
         <v>111</v>
       </c>
       <c r="B94" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C94" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.2">
@@ -4021,10 +4021,10 @@
         <v>112</v>
       </c>
       <c r="B95" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C95" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.2">
@@ -4032,10 +4032,10 @@
         <v>113</v>
       </c>
       <c r="B96" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C96" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.2">
@@ -4043,10 +4043,10 @@
         <v>114</v>
       </c>
       <c r="B97" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C97" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.2">
@@ -4065,10 +4065,10 @@
         <v>117</v>
       </c>
       <c r="B99" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C99" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.2">
@@ -4076,10 +4076,10 @@
         <v>119</v>
       </c>
       <c r="B100" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C100" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
@@ -4087,10 +4087,10 @@
         <v>120</v>
       </c>
       <c r="B101" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C101" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
@@ -4098,10 +4098,10 @@
         <v>121</v>
       </c>
       <c r="B102" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C102" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.2">
@@ -4120,10 +4120,10 @@
         <v>126</v>
       </c>
       <c r="B104" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C104" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.2">
@@ -4131,10 +4131,10 @@
         <v>127</v>
       </c>
       <c r="B105" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C105" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.2">
@@ -4142,10 +4142,10 @@
         <v>131</v>
       </c>
       <c r="B106" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C106" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.2">
@@ -4153,10 +4153,10 @@
         <v>133</v>
       </c>
       <c r="B107" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C107" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.2">
@@ -4164,10 +4164,10 @@
         <v>134</v>
       </c>
       <c r="B108" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C108" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.2">
@@ -4175,10 +4175,10 @@
         <v>136</v>
       </c>
       <c r="B109" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C109" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.2">
@@ -4186,10 +4186,10 @@
         <v>141</v>
       </c>
       <c r="B110" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C110" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.2">
@@ -4197,10 +4197,10 @@
         <v>142</v>
       </c>
       <c r="B111" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C111" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.2">
@@ -4219,10 +4219,10 @@
         <v>145</v>
       </c>
       <c r="B113" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C113" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.2">
@@ -4230,10 +4230,10 @@
         <v>147</v>
       </c>
       <c r="B114" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C114" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.2">
@@ -4241,10 +4241,10 @@
         <v>150</v>
       </c>
       <c r="B115" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C115" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.2">
@@ -4252,10 +4252,10 @@
         <v>154</v>
       </c>
       <c r="B116" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C116" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.2">
@@ -4263,10 +4263,10 @@
         <v>157</v>
       </c>
       <c r="B117" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C117" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.2">
@@ -4274,10 +4274,10 @@
         <v>161</v>
       </c>
       <c r="B118" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C118" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.2">
@@ -4285,10 +4285,10 @@
         <v>163</v>
       </c>
       <c r="B119" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C119" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.2">
@@ -4296,10 +4296,10 @@
         <v>164</v>
       </c>
       <c r="B120" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C120" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.2">
@@ -4307,10 +4307,10 @@
         <v>166</v>
       </c>
       <c r="B121" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C121" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.2">
@@ -4318,10 +4318,10 @@
         <v>200</v>
       </c>
       <c r="B122" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C122" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.2">
@@ -4329,10 +4329,10 @@
         <v>201</v>
       </c>
       <c r="B123" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C123" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.2">
@@ -4340,10 +4340,10 @@
         <v>202</v>
       </c>
       <c r="B124" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C124" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.2">
@@ -4351,10 +4351,10 @@
         <v>203</v>
       </c>
       <c r="B125" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C125" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.2">
@@ -4362,10 +4362,10 @@
         <v>221</v>
       </c>
       <c r="B126" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C126" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.2">
@@ -4373,10 +4373,10 @@
         <v>222</v>
       </c>
       <c r="B127" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C127" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.2">
@@ -4384,10 +4384,10 @@
         <v>223</v>
       </c>
       <c r="B128" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C128" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.2">
@@ -4395,10 +4395,10 @@
         <v>233</v>
       </c>
       <c r="B129" t="s">
+        <v>327</v>
+      </c>
+      <c r="C129" t="s">
         <v>328</v>
-      </c>
-      <c r="C129" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.2">
@@ -4406,10 +4406,10 @@
         <v>234</v>
       </c>
       <c r="B130" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C130" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.2">
@@ -4417,10 +4417,10 @@
         <v>235</v>
       </c>
       <c r="B131" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C131" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.2">
@@ -4439,10 +4439,10 @@
         <v>238</v>
       </c>
       <c r="B133" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C133" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.2">
@@ -4450,10 +4450,10 @@
         <v>240</v>
       </c>
       <c r="B134" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C134" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.2">
@@ -4461,10 +4461,10 @@
         <v>245</v>
       </c>
       <c r="B135" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C135" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.2">
@@ -4472,10 +4472,10 @@
         <v>246</v>
       </c>
       <c r="B136" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C136" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.2">
@@ -4483,10 +4483,10 @@
         <v>254</v>
       </c>
       <c r="B137" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C137" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.2">
@@ -4494,10 +4494,10 @@
         <v>266</v>
       </c>
       <c r="B138" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C138" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.2">
@@ -4505,10 +4505,10 @@
         <v>267</v>
       </c>
       <c r="B139" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C139" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.2">
@@ -4516,10 +4516,10 @@
         <v>268</v>
       </c>
       <c r="B140" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C140" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.2">
@@ -4527,10 +4527,10 @@
         <v>350</v>
       </c>
       <c r="B141" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C141" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.2">
@@ -4538,10 +4538,10 @@
         <v>360</v>
       </c>
       <c r="B142" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C142" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.2">
@@ -4549,10 +4549,10 @@
         <v>412</v>
       </c>
       <c r="B143" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C143" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.2">
@@ -4560,10 +4560,10 @@
         <v>420</v>
       </c>
       <c r="B144" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C144" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.2">
@@ -4571,10 +4571,10 @@
         <v>421</v>
       </c>
       <c r="B145" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C145" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.2">
@@ -4582,10 +4582,10 @@
         <v>427</v>
       </c>
       <c r="B146" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C146" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.2">
@@ -4593,10 +4593,10 @@
         <v>429</v>
       </c>
       <c r="B147" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C147" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.2">
@@ -4604,10 +4604,10 @@
         <v>432</v>
       </c>
       <c r="B148" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C148" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.2">
@@ -4615,10 +4615,10 @@
         <v>497</v>
       </c>
       <c r="B149" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C149" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.2">
@@ -4626,10 +4626,10 @@
         <v>498</v>
       </c>
       <c r="B150" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C150" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.2">
@@ -4637,10 +4637,10 @@
         <v>516</v>
       </c>
       <c r="B151" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C151" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.2">
@@ -4648,10 +4648,10 @@
         <v>517</v>
       </c>
       <c r="B152" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C152" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.2">
@@ -4659,10 +4659,10 @@
         <v>518</v>
       </c>
       <c r="B153" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C153" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.2">
@@ -4670,10 +4670,10 @@
         <v>523</v>
       </c>
       <c r="B154" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C154" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.2">
@@ -4681,10 +4681,10 @@
         <v>526</v>
       </c>
       <c r="B155" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C155" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.2">
@@ -4692,10 +4692,10 @@
         <v>555</v>
       </c>
       <c r="B156" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C156" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.2">
@@ -4703,10 +4703,10 @@
         <v>711</v>
       </c>
       <c r="B157" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C157" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.2">
@@ -4714,10 +4714,10 @@
         <v>777</v>
       </c>
       <c r="B158" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C158" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.2">
@@ -4725,10 +4725,10 @@
         <v>875</v>
       </c>
       <c r="B159" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C159" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.2">
@@ -4736,10 +4736,10 @@
         <v>876</v>
       </c>
       <c r="B160" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C160" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.2">
@@ -4747,10 +4747,10 @@
         <v>887</v>
       </c>
       <c r="B161" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C161" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.2">
@@ -4758,10 +4758,10 @@
         <v>888</v>
       </c>
       <c r="B162" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C162" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.2">
@@ -4769,10 +4769,10 @@
         <v>895</v>
       </c>
       <c r="B163" t="s">
+        <v>318</v>
+      </c>
+      <c r="C163" t="s">
         <v>319</v>
-      </c>
-      <c r="C163" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.2">
@@ -4780,10 +4780,10 @@
         <v>897</v>
       </c>
       <c r="B164" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C164" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.2">
@@ -4791,10 +4791,10 @@
         <v>901</v>
       </c>
       <c r="B165" t="s">
+        <v>334</v>
+      </c>
+      <c r="C165" t="s">
         <v>335</v>
-      </c>
-      <c r="C165" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.2">
@@ -4802,10 +4802,10 @@
         <v>902</v>
       </c>
       <c r="B166" t="s">
+        <v>321</v>
+      </c>
+      <c r="C166" t="s">
         <v>322</v>
-      </c>
-      <c r="C166" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.2">
@@ -4813,10 +4813,10 @@
         <v>910</v>
       </c>
       <c r="B167" t="s">
+        <v>329</v>
+      </c>
+      <c r="C167" t="s">
         <v>330</v>
-      </c>
-      <c r="C167" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.2">
@@ -4824,10 +4824,10 @@
         <v>950</v>
       </c>
       <c r="B168" t="s">
+        <v>323</v>
+      </c>
+      <c r="C168" t="s">
         <v>324</v>
-      </c>
-      <c r="C168" t="s">
-        <v>325</v>
       </c>
     </row>
   </sheetData>

</xml_diff>